<commit_message>
baseline models on marcos covs, experimenting with all covs, visualization, hawkes model
</commit_message>
<xml_diff>
--- a/Data/EventData/SDGE_2021.xlsx
+++ b/Data/EventData/SDGE_2021.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sempra-my.sharepoint.com/personal/cstaylor_semprautilities_com/Documents/1_Work/Regulatory/Cases/3. D.14-02-015 Reportable Ignitions Annual Report  (Due April 1)/Reports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dread\Downloads\Wildfire-Point-Process\Data\EventData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="11_F0E53992E3A71056894F9F7593A2DE1F5E8B8B4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA0E9A83-6D5D-4D46-8735-DAC0957C55E7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EFAA1D-CAFF-4E5B-B765-844A9E520351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interactive (2021)" sheetId="3" r:id="rId1"/>
@@ -515,7 +515,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="158">
   <si>
     <t>Utility Name</t>
   </si>
@@ -737,9 +737,6 @@
     <t>Vandalism/Theft</t>
   </si>
   <si>
-    <t>18;26</t>
-  </si>
-  <si>
     <t>372756J</t>
   </si>
   <si>
@@ -806,9 +803,6 @@
     <t>P372261</t>
   </si>
   <si>
-    <t>This report includes SDG&amp;E’s preliminary assessment of the cause of the ignition; the cause of any ignition may remain subject to ongoing investigation by the appropriate fire investigation agency</t>
-  </si>
-  <si>
     <t>BVES</t>
   </si>
   <si>
@@ -996,21 +990,18 @@
   </si>
   <si>
     <t>Voltage Regulator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blacked-out cells means N/A </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="m/d/yy;@"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
     <numFmt numFmtId="166" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1062,14 +1053,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1154,14 +1139,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="23">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -1422,38 +1401,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1631,49 +1583,6 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="15" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="15" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1759,21 +1668,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
@@ -1791,7 +1686,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor indexed="8"/>
+          <bgColor theme="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1826,33 +1721,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor indexed="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor indexed="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor indexed="8"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{C8F1227E-FD18-4E0E-ACB1-134517E37861}"/>
+  </tableStyles>
   <colors>
     <mruColors>
       <color rgb="FFCCFFFF"/>
@@ -1872,9 +1748,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1912,9 +1788,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1947,26 +1823,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1999,26 +1858,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2195,7 +2037,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:W27"/>
   <sheetFormatPr defaultColWidth="9.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2" customWidth="1"/>
@@ -2225,44 +2067,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="99" t="s">
+      <c r="B1" s="80"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="102" t="s">
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="103"/>
-      <c r="J1" s="104"/>
-      <c r="K1" s="105" t="s">
+      <c r="I1" s="88"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="90" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="106"/>
-      <c r="M1" s="106"/>
-      <c r="N1" s="106"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="108" t="s">
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="92"/>
+      <c r="P1" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="109"/>
-      <c r="R1" s="110"/>
-      <c r="S1" s="92" t="s">
+      <c r="Q1" s="94"/>
+      <c r="R1" s="95"/>
+      <c r="S1" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="93"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
+      <c r="T1" s="78"/>
+      <c r="U1" s="79"/>
+      <c r="V1" s="79"/>
+      <c r="W1" s="79"/>
     </row>
     <row r="2" spans="1:23" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="98"/>
+      <c r="A2" s="83"/>
       <c r="B2" s="9" t="s">
         <v>6</v>
       </c>
@@ -2305,7 +2147,7 @@
       <c r="O2" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="84" t="s">
+      <c r="P2" s="69" t="s">
         <v>20</v>
       </c>
       <c r="Q2" s="20" t="s">
@@ -2338,7 +2180,7 @@
         <v>44255</v>
       </c>
       <c r="C3" s="26">
-        <v>1300.5833333333333</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="D3" s="27">
         <v>33.436999999999998</v>
@@ -2362,8 +2204,8 @@
       <c r="K3" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="91"/>
-      <c r="M3" s="87" t="s">
+      <c r="L3" s="76"/>
+      <c r="M3" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N3" s="35" t="s">
@@ -2372,7 +2214,7 @@
       <c r="O3" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="P3" s="85" t="s">
+      <c r="P3" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q3" s="37">
@@ -2427,8 +2269,8 @@
       <c r="K4" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="L4" s="91"/>
-      <c r="M4" s="87" t="s">
+      <c r="L4" s="76"/>
+      <c r="M4" s="72" t="s">
         <v>40</v>
       </c>
       <c r="N4" s="35" t="s">
@@ -2437,7 +2279,7 @@
       <c r="O4" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P4" s="85" t="s">
+      <c r="P4" s="70" t="s">
         <v>42</v>
       </c>
       <c r="Q4" s="37"/>
@@ -2488,8 +2330,8 @@
       <c r="K5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="L5" s="91"/>
-      <c r="M5" s="87" t="s">
+      <c r="L5" s="76"/>
+      <c r="M5" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N5" s="35" t="s">
@@ -2498,7 +2340,7 @@
       <c r="O5" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P5" s="85" t="s">
+      <c r="P5" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q5" s="37">
@@ -2553,8 +2395,8 @@
       <c r="K6" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="87" t="s">
+      <c r="L6" s="76"/>
+      <c r="M6" s="72" t="s">
         <v>53</v>
       </c>
       <c r="N6" s="35" t="s">
@@ -2563,7 +2405,7 @@
       <c r="O6" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P6" s="85" t="s">
+      <c r="P6" s="70" t="s">
         <v>42</v>
       </c>
       <c r="Q6" s="37"/>
@@ -2612,8 +2454,8 @@
         <v>54</v>
       </c>
       <c r="K7" s="34"/>
-      <c r="L7" s="91"/>
-      <c r="M7" s="87" t="s">
+      <c r="L7" s="76"/>
+      <c r="M7" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N7" s="35" t="s">
@@ -2622,7 +2464,7 @@
       <c r="O7" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P7" s="85" t="s">
+      <c r="P7" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q7" s="37">
@@ -2677,8 +2519,8 @@
         <v>55</v>
       </c>
       <c r="K8" s="34"/>
-      <c r="L8" s="91"/>
-      <c r="M8" s="87" t="s">
+      <c r="L8" s="76"/>
+      <c r="M8" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N8" s="35" t="s">
@@ -2687,7 +2529,7 @@
       <c r="O8" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P8" s="85" t="s">
+      <c r="P8" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q8" s="37">
@@ -2742,8 +2584,8 @@
       <c r="K9" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="L9" s="91"/>
-      <c r="M9" s="87" t="s">
+      <c r="L9" s="76"/>
+      <c r="M9" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N9" s="35" t="s">
@@ -2752,7 +2594,7 @@
       <c r="O9" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P9" s="85" t="s">
+      <c r="P9" s="70" t="s">
         <v>42</v>
       </c>
       <c r="Q9" s="37"/>
@@ -2801,8 +2643,8 @@
       <c r="K10" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="L10" s="91"/>
-      <c r="M10" s="87" t="s">
+      <c r="L10" s="76"/>
+      <c r="M10" s="72" t="s">
         <v>53</v>
       </c>
       <c r="N10" s="35" t="s">
@@ -2811,7 +2653,7 @@
       <c r="O10" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P10" s="85" t="s">
+      <c r="P10" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q10" s="37">
@@ -2868,8 +2710,8 @@
       <c r="K11" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="L11" s="91"/>
-      <c r="M11" s="87" t="s">
+      <c r="L11" s="76"/>
+      <c r="M11" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N11" s="35" t="s">
@@ -2878,7 +2720,7 @@
       <c r="O11" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P11" s="85" t="s">
+      <c r="P11" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q11" s="37">
@@ -2933,8 +2775,8 @@
       <c r="K12" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="L12" s="91"/>
-      <c r="M12" s="87" t="s">
+      <c r="L12" s="76"/>
+      <c r="M12" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N12" s="35" t="s">
@@ -2943,7 +2785,7 @@
       <c r="O12" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P12" s="85" t="s">
+      <c r="P12" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q12" s="37">
@@ -2996,8 +2838,8 @@
       <c r="K13" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="L13" s="91"/>
-      <c r="M13" s="87" t="s">
+      <c r="L13" s="76"/>
+      <c r="M13" s="72" t="s">
         <v>66</v>
       </c>
       <c r="N13" s="35" t="s">
@@ -3006,7 +2848,7 @@
       <c r="O13" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P13" s="85" t="s">
+      <c r="P13" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q13" s="37">
@@ -3062,10 +2904,10 @@
       <c r="K14" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="L14" s="91" t="s">
+      <c r="L14" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="M14" s="87" t="s">
+      <c r="M14" s="72" t="s">
         <v>66</v>
       </c>
       <c r="N14" s="35" t="s">
@@ -3074,7 +2916,7 @@
       <c r="O14" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P14" s="85" t="s">
+      <c r="P14" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q14" s="37">
@@ -3129,8 +2971,8 @@
       <c r="K15" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="L15" s="91"/>
-      <c r="M15" s="87" t="s">
+      <c r="L15" s="76"/>
+      <c r="M15" s="72" t="s">
         <v>66</v>
       </c>
       <c r="N15" s="35" t="s">
@@ -3139,7 +2981,7 @@
       <c r="O15" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P15" s="85" t="s">
+      <c r="P15" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q15" s="37">
@@ -3167,8 +3009,8 @@
       <c r="B16" s="42">
         <v>44391</v>
       </c>
-      <c r="C16" s="26" t="s">
-        <v>73</v>
+      <c r="C16" s="26">
+        <v>0.7680555555555556</v>
       </c>
       <c r="D16" s="28">
         <v>32.503799999999998</v>
@@ -3190,10 +3032,10 @@
       </c>
       <c r="J16" s="33"/>
       <c r="K16" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="L16" s="91"/>
-      <c r="M16" s="87" t="s">
+        <v>73</v>
+      </c>
+      <c r="L16" s="76"/>
+      <c r="M16" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N16" s="35" t="s">
@@ -3202,7 +3044,7 @@
       <c r="O16" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P16" s="85" t="s">
+      <c r="P16" s="70" t="s">
         <v>42</v>
       </c>
       <c r="Q16" s="37"/>
@@ -3249,10 +3091,10 @@
       </c>
       <c r="J17" s="33"/>
       <c r="K17" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="L17" s="91"/>
-      <c r="M17" s="87" t="s">
+        <v>74</v>
+      </c>
+      <c r="L17" s="76"/>
+      <c r="M17" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N17" s="35" t="s">
@@ -3261,7 +3103,7 @@
       <c r="O17" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P17" s="85" t="s">
+      <c r="P17" s="70" t="s">
         <v>42</v>
       </c>
       <c r="Q17" s="37"/>
@@ -3273,7 +3115,7 @@
       <c r="U17" s="41"/>
       <c r="V17" s="41"/>
       <c r="W17" s="41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
@@ -3299,19 +3141,19 @@
         <v>28</v>
       </c>
       <c r="H18" s="55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I18" s="56" t="s">
         <v>50</v>
       </c>
       <c r="J18" s="57" t="s">
+        <v>77</v>
+      </c>
+      <c r="K18" s="58" t="s">
         <v>78</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>79</v>
-      </c>
-      <c r="L18" s="91"/>
-      <c r="M18" s="88" t="s">
+      <c r="L18" s="76"/>
+      <c r="M18" s="73" t="s">
         <v>32</v>
       </c>
       <c r="N18" s="59" t="s">
@@ -3320,13 +3162,13 @@
       <c r="O18" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P18" s="86" t="s">
+      <c r="P18" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q18" s="89">
+      <c r="Q18" s="74">
         <v>44401</v>
       </c>
-      <c r="R18" s="90">
+      <c r="R18" s="75">
         <v>0.6381944444444444</v>
       </c>
       <c r="S18" s="61" t="s">
@@ -3366,19 +3208,19 @@
         <v>28</v>
       </c>
       <c r="H19" s="55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I19" s="56" t="s">
         <v>50</v>
       </c>
       <c r="J19" s="57" t="s">
+        <v>79</v>
+      </c>
+      <c r="K19" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="K19" s="58" t="s">
-        <v>81</v>
-      </c>
-      <c r="L19" s="91"/>
-      <c r="M19" s="88" t="s">
+      <c r="L19" s="76"/>
+      <c r="M19" s="73" t="s">
         <v>32</v>
       </c>
       <c r="N19" s="59" t="s">
@@ -3387,17 +3229,17 @@
       <c r="O19" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P19" s="86" t="s">
+      <c r="P19" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q19" s="89">
+      <c r="Q19" s="74">
         <v>44405</v>
       </c>
-      <c r="R19" s="90">
+      <c r="R19" s="75">
         <v>0.57708333333333328</v>
       </c>
       <c r="S19" s="61" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T19" s="45"/>
       <c r="U19" s="63"/>
@@ -3438,11 +3280,11 @@
         <v>67</v>
       </c>
       <c r="K20" s="58" t="s">
+        <v>82</v>
+      </c>
+      <c r="L20" s="76"/>
+      <c r="M20" s="73" t="s">
         <v>83</v>
-      </c>
-      <c r="L20" s="91"/>
-      <c r="M20" s="88" t="s">
-        <v>84</v>
       </c>
       <c r="N20" s="59" t="s">
         <v>41</v>
@@ -3450,13 +3292,13 @@
       <c r="O20" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P20" s="86" t="s">
+      <c r="P20" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q20" s="89">
+      <c r="Q20" s="74">
         <v>44406</v>
       </c>
-      <c r="R20" s="90">
+      <c r="R20" s="75">
         <v>0.7715277777777777</v>
       </c>
       <c r="S20" s="61" t="s">
@@ -3502,14 +3344,14 @@
         <v>50</v>
       </c>
       <c r="J21" s="57" t="s">
+        <v>84</v>
+      </c>
+      <c r="K21" s="58" t="s">
         <v>85</v>
       </c>
-      <c r="K21" s="58" t="s">
-        <v>86</v>
-      </c>
-      <c r="L21" s="91"/>
-      <c r="M21" s="88" t="s">
-        <v>84</v>
+      <c r="L21" s="76"/>
+      <c r="M21" s="73" t="s">
+        <v>83</v>
       </c>
       <c r="N21" s="59" t="s">
         <v>41</v>
@@ -3517,21 +3359,21 @@
       <c r="O21" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P21" s="86" t="s">
+      <c r="P21" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="Q21" s="89"/>
-      <c r="R21" s="90"/>
+      <c r="Q21" s="74"/>
+      <c r="R21" s="75"/>
       <c r="S21" s="61" t="s">
         <v>48</v>
       </c>
       <c r="T21" s="45" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="U21" s="63"/>
       <c r="V21" s="63"/>
       <c r="W21" s="63" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3566,10 +3408,10 @@
         <v>55</v>
       </c>
       <c r="K22" s="58" t="s">
-        <v>88</v>
-      </c>
-      <c r="L22" s="91"/>
-      <c r="M22" s="88" t="s">
+        <v>87</v>
+      </c>
+      <c r="L22" s="76"/>
+      <c r="M22" s="73" t="s">
         <v>32</v>
       </c>
       <c r="N22" s="59" t="s">
@@ -3578,13 +3420,13 @@
       <c r="O22" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P22" s="86" t="s">
+      <c r="P22" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q22" s="89">
+      <c r="Q22" s="74">
         <v>44415</v>
       </c>
-      <c r="R22" s="90">
+      <c r="R22" s="75">
         <v>0.46388888888888885</v>
       </c>
       <c r="S22" s="61" t="s">
@@ -3633,10 +3475,10 @@
         <v>59</v>
       </c>
       <c r="K23" s="58" t="s">
-        <v>89</v>
-      </c>
-      <c r="L23" s="91"/>
-      <c r="M23" s="88" t="s">
+        <v>88</v>
+      </c>
+      <c r="L23" s="76"/>
+      <c r="M23" s="73" t="s">
         <v>32</v>
       </c>
       <c r="N23" s="59" t="s">
@@ -3645,20 +3487,20 @@
       <c r="O23" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P23" s="86" t="s">
+      <c r="P23" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q23" s="89">
+      <c r="Q23" s="74">
         <v>44433</v>
       </c>
-      <c r="R23" s="90">
+      <c r="R23" s="75">
         <v>0.22569444444444445</v>
       </c>
       <c r="S23" s="61" t="s">
         <v>48</v>
       </c>
       <c r="T23" s="45" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="U23" s="63"/>
       <c r="V23" s="63"/>
@@ -3674,7 +3516,7 @@
         <v>44470</v>
       </c>
       <c r="C24" s="65">
-        <v>1203</v>
+        <v>0</v>
       </c>
       <c r="D24" s="51">
         <v>32.692329999999998</v>
@@ -3689,19 +3531,19 @@
         <v>28</v>
       </c>
       <c r="H24" s="55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I24" s="56" t="s">
         <v>50</v>
       </c>
       <c r="J24" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="K24" s="58" t="s">
         <v>90</v>
       </c>
-      <c r="K24" s="58" t="s">
-        <v>91</v>
-      </c>
-      <c r="L24" s="91"/>
-      <c r="M24" s="88" t="s">
+      <c r="L24" s="76"/>
+      <c r="M24" s="73" t="s">
         <v>40</v>
       </c>
       <c r="N24" s="59" t="s">
@@ -3710,13 +3552,13 @@
       <c r="O24" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P24" s="86" t="s">
+      <c r="P24" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q24" s="89">
+      <c r="Q24" s="74">
         <v>44470</v>
       </c>
-      <c r="R24" s="90">
+      <c r="R24" s="75">
         <v>1202</v>
       </c>
       <c r="S24" s="61" t="s">
@@ -3759,14 +3601,14 @@
         <v>29</v>
       </c>
       <c r="I25" s="56" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J25" s="57"/>
       <c r="K25" s="58" t="s">
-        <v>93</v>
-      </c>
-      <c r="L25" s="91"/>
-      <c r="M25" s="88" t="s">
+        <v>92</v>
+      </c>
+      <c r="L25" s="76"/>
+      <c r="M25" s="73" t="s">
         <v>32</v>
       </c>
       <c r="N25" s="59" t="s">
@@ -3775,13 +3617,13 @@
       <c r="O25" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P25" s="86" t="s">
+      <c r="P25" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q25" s="89">
+      <c r="Q25" s="74">
         <v>44530</v>
       </c>
-      <c r="R25" s="90">
+      <c r="R25" s="75">
         <v>0.4069444444444445</v>
       </c>
       <c r="S25" s="61" t="s">
@@ -3806,7 +3648,7 @@
         <v>44533</v>
       </c>
       <c r="C26" s="26">
-        <v>1048.5138888888889</v>
+        <v>0.51388888888888884</v>
       </c>
       <c r="D26" s="51">
         <v>32.567999999999998</v>
@@ -3830,10 +3672,10 @@
         <v>59</v>
       </c>
       <c r="K26" s="58" t="s">
-        <v>94</v>
-      </c>
-      <c r="L26" s="91"/>
-      <c r="M26" s="88" t="s">
+        <v>93</v>
+      </c>
+      <c r="L26" s="76"/>
+      <c r="M26" s="73" t="s">
         <v>32</v>
       </c>
       <c r="N26" s="59" t="s">
@@ -3842,13 +3684,13 @@
       <c r="O26" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="P26" s="86" t="s">
+      <c r="P26" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="Q26" s="89">
+      <c r="Q26" s="74">
         <v>44533</v>
       </c>
-      <c r="R26" s="90">
+      <c r="R26" s="75">
         <v>1048.5138888888889</v>
       </c>
       <c r="S26" s="61" t="s">
@@ -3894,13 +3736,13 @@
         <v>50</v>
       </c>
       <c r="J27" s="33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K27" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="L27" s="91"/>
-      <c r="M27" s="87" t="s">
+        <v>94</v>
+      </c>
+      <c r="L27" s="76"/>
+      <c r="M27" s="72" t="s">
         <v>66</v>
       </c>
       <c r="N27" s="35" t="s">
@@ -3909,7 +3751,7 @@
       <c r="O27" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="P27" s="85" t="s">
+      <c r="P27" s="70" t="s">
         <v>35</v>
       </c>
       <c r="Q27" s="37">
@@ -3922,117 +3764,13 @@
         <v>48</v>
       </c>
       <c r="T27" s="45" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="U27" s="41"/>
       <c r="V27" s="41"/>
       <c r="W27" s="41" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="28" spans="1:23" ht="8.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="69"/>
-      <c r="B28" s="70"/>
-      <c r="C28" s="71"/>
-      <c r="D28" s="72"/>
-      <c r="E28" s="72"/>
-      <c r="F28" s="73"/>
-      <c r="G28" s="73"/>
-      <c r="H28" s="72"/>
-      <c r="I28" s="72"/>
-      <c r="J28" s="72"/>
-      <c r="K28" s="73"/>
-      <c r="L28" s="73"/>
-      <c r="M28" s="74"/>
-      <c r="N28" s="72"/>
-      <c r="O28" s="72"/>
-      <c r="P28" s="72"/>
-      <c r="Q28" s="73"/>
-      <c r="R28" s="73"/>
-      <c r="S28" s="72"/>
-      <c r="T28" s="72"/>
-      <c r="U28" s="72"/>
-      <c r="V28" s="72"/>
-      <c r="W28" s="75"/>
-    </row>
-    <row r="29" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="76" t="s">
-        <v>160</v>
-      </c>
-      <c r="B29" s="70"/>
-      <c r="C29" s="71"/>
-      <c r="D29" s="72"/>
-      <c r="E29" s="72"/>
-      <c r="F29" s="73"/>
-      <c r="G29" s="73"/>
-      <c r="H29" s="72"/>
-      <c r="I29" s="72"/>
-      <c r="J29" s="72"/>
-      <c r="K29" s="73"/>
-      <c r="L29" s="73"/>
-      <c r="M29" s="74"/>
-      <c r="N29" s="72"/>
-      <c r="O29" s="72"/>
-      <c r="P29" s="72"/>
-      <c r="Q29" s="73"/>
-      <c r="R29" s="73"/>
-      <c r="S29" s="72"/>
-      <c r="T29" s="72"/>
-      <c r="U29" s="72"/>
-      <c r="V29" s="72"/>
-      <c r="W29" s="75"/>
-    </row>
-    <row r="30" spans="1:23" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="76"/>
-      <c r="B30" s="70"/>
-      <c r="C30" s="71"/>
-      <c r="D30" s="72"/>
-      <c r="E30" s="72"/>
-      <c r="F30" s="73"/>
-      <c r="G30" s="73"/>
-      <c r="H30" s="72"/>
-      <c r="I30" s="72"/>
-      <c r="J30" s="72"/>
-      <c r="K30" s="73"/>
-      <c r="L30" s="73"/>
-      <c r="M30" s="74"/>
-      <c r="N30" s="72"/>
-      <c r="O30" s="72"/>
-      <c r="P30" s="72"/>
-      <c r="Q30" s="73"/>
-      <c r="R30" s="73"/>
-      <c r="S30" s="72"/>
-      <c r="T30" s="72"/>
-      <c r="U30" s="72"/>
-      <c r="V30" s="72"/>
-      <c r="W30" s="75"/>
-    </row>
-    <row r="31" spans="1:23" s="83" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A31" s="77" t="s">
-        <v>96</v>
-      </c>
-      <c r="B31" s="78"/>
-      <c r="C31" s="79"/>
-      <c r="D31" s="80"/>
-      <c r="E31" s="80"/>
-      <c r="F31" s="81"/>
-      <c r="G31" s="81"/>
-      <c r="H31" s="80"/>
-      <c r="I31" s="80"/>
-      <c r="J31" s="80"/>
-      <c r="K31" s="81"/>
-      <c r="L31" s="81"/>
-      <c r="M31" s="80"/>
-      <c r="N31" s="80"/>
-      <c r="O31" s="80"/>
-      <c r="P31" s="80"/>
-      <c r="Q31" s="81"/>
-      <c r="R31" s="81"/>
-      <c r="S31" s="80"/>
-      <c r="T31" s="80"/>
-      <c r="U31" s="80"/>
-      <c r="V31" s="80"/>
-      <c r="W31" s="82"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -4045,69 +3783,44 @@
     <mergeCell ref="K1:O1"/>
     <mergeCell ref="P1:R1"/>
   </mergeCells>
-  <conditionalFormatting sqref="J3:J25 J27">
-    <cfRule type="expression" dxfId="12" priority="28" stopIfTrue="1">
+  <conditionalFormatting sqref="J3:J27">
+    <cfRule type="expression" dxfId="7" priority="2" stopIfTrue="1">
       <formula>IF(I3&lt;&gt;"Fire Agency",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U3:U25 U27">
-    <cfRule type="expression" dxfId="11" priority="29" stopIfTrue="1">
+  <conditionalFormatting sqref="L3:L17">
+    <cfRule type="expression" dxfId="6" priority="26" stopIfTrue="1">
+      <formula>IF($O3&lt;&gt;"Overhead",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L18">
+    <cfRule type="expression" dxfId="5" priority="31" stopIfTrue="1">
+      <formula>IF($O21&lt;&gt;"Overhead",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L19:L27">
+    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
+      <formula>IF($O19&lt;&gt;"Overhead",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q3:R27">
+    <cfRule type="expression" dxfId="3" priority="7" stopIfTrue="1">
+      <formula>IF($P3&lt;&gt;"Yes",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T3:T27">
+    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
+      <formula>IF(S3&lt;&gt;"Equipment/Facility Failure",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U3:U27">
+    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
       <formula>IF(S3&lt;&gt;"Contact From Object",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q3:R25 Q27:R27">
-    <cfRule type="expression" dxfId="10" priority="30" stopIfTrue="1">
-      <formula>IF($P3&lt;&gt;"Yes",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V3:V25 V27">
-    <cfRule type="expression" dxfId="9" priority="27" stopIfTrue="1">
+  <conditionalFormatting sqref="V3:V27">
+    <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">
       <formula>IF(S3&lt;&gt;"Contact From Object",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L19:L25 L3:L17">
-    <cfRule type="expression" dxfId="8" priority="26" stopIfTrue="1">
-      <formula>IF($O3&lt;&gt;"Overhead",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T3:T25 T27">
-    <cfRule type="expression" dxfId="7" priority="25" stopIfTrue="1">
-      <formula>IF(S3&lt;&gt;"Equipment/Facility Failure",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L18">
-    <cfRule type="expression" dxfId="6" priority="31" stopIfTrue="1">
-      <formula>IF($O21&lt;&gt;"Overhead",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J26">
-    <cfRule type="expression" dxfId="5" priority="2" stopIfTrue="1">
-      <formula>IF(I26&lt;&gt;"Fire Agency",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U26">
-    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
-      <formula>IF(S26&lt;&gt;"Contact From Object",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q26:R26">
-    <cfRule type="expression" dxfId="3" priority="7" stopIfTrue="1">
-      <formula>IF($P26&lt;&gt;"Yes",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V26">
-    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
-      <formula>IF(S26&lt;&gt;"Contact From Object",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T26">
-    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
-      <formula>IF(S26&lt;&gt;"Equipment/Facility Failure",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L26:L27">
-    <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
-      <formula>IF($O26&lt;&gt;"Overhead",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="13">
@@ -4185,25 +3898,25 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>70</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>36</v>
@@ -4218,33 +3931,33 @@
         <v>29</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>70</v>
       </c>
       <c r="N2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="T2" s="1">
         <v>1</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>44</v>
@@ -4274,7 +3987,7 @@
         <v>42</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L3" s="1" t="s">
         <v>37</v>
@@ -4283,28 +3996,28 @@
         <v>41</v>
       </c>
       <c r="N3" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="T3" s="1">
         <f>T2+1</f>
         <v>2</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>27</v>
@@ -4313,13 +4026,13 @@
         <v>30</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>115</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>44</v>
@@ -4328,43 +4041,43 @@
         <v>44</v>
       </c>
       <c r="K4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="M4" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="N4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="T4" s="1">
         <f t="shared" ref="T4:T18" si="0">T3+1</f>
         <v>3</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>49</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>48</v>
@@ -4376,28 +4089,28 @@
         <v>38</v>
       </c>
       <c r="K5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="T5" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>46</v>
@@ -4406,37 +4119,37 @@
         <v>44</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>49</v>
       </c>
       <c r="K6" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="S6" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>135</v>
       </c>
       <c r="T6" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>64</v>
@@ -4445,26 +4158,26 @@
         <v>44</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K7" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S7" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="T7" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
@@ -4472,7 +4185,7 @@
         <v>26</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>33</v>
@@ -4481,16 +4194,16 @@
         <v>49</v>
       </c>
       <c r="K8" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="P8" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="S8" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="T8" s="1">
         <f t="shared" si="0"/>
@@ -4502,16 +4215,16 @@
         <v>72</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>44</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="T9" s="1">
         <f t="shared" si="0"/>
@@ -4523,13 +4236,13 @@
         <v>57</v>
       </c>
       <c r="K10" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="S10" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="T10" s="1">
         <f t="shared" si="0"/>
@@ -4539,10 +4252,10 @@
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="G11" s="8"/>
       <c r="M11" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="T11" s="1">
         <f t="shared" si="0"/>
@@ -4552,10 +4265,10 @@
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="G12" s="8"/>
       <c r="M12" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="T12" s="1">
         <f t="shared" si="0"/>
@@ -4565,10 +4278,10 @@
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="G13" s="8"/>
       <c r="M13" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="T13" s="1">
         <f t="shared" si="0"/>
@@ -4577,10 +4290,10 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="G14" s="8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="T14" s="1">
         <f t="shared" si="0"/>
@@ -4610,7 +4323,7 @@
     <row r="17" spans="7:20" x14ac:dyDescent="0.3">
       <c r="G17" s="8"/>
       <c r="M17" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="T17" s="1">
         <f t="shared" si="0"/>
@@ -4633,18 +4346,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="c1ca76c8-b577-4424-b1c5-5c92107fcf49">
-      <UserInfo>
-        <DisplayName>Cui, Ye (Contractor)</DisplayName>
-        <AccountId>122</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <SharedWithDetails xmlns="c1ca76c8-b577-4424-b1c5-5c92107fcf49">{"i:0#.f|membership|lycui@sdgecontractor.com":{"DateTime":"\/Date(1596649890242)\/","LoginName":"rveihl@semprautilities.com"}}</SharedWithDetails>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4878,20 +4585,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="c1ca76c8-b577-4424-b1c5-5c92107fcf49">
+      <UserInfo>
+        <DisplayName>Cui, Ye (Contractor)</DisplayName>
+        <AccountId>122</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <SharedWithDetails xmlns="c1ca76c8-b577-4424-b1c5-5c92107fcf49">{"i:0#.f|membership|lycui@sdgecontractor.com":{"DateTime":"\/Date(1596649890242)\/","LoginName":"rveihl@semprautilities.com"}}</SharedWithDetails>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E29F4A5-09ED-4CF7-BCF2-7F7E65809C74}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B0F4E8F-EADE-4687-BD92-9F44E749F726}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c1ca76c8-b577-4424-b1c5-5c92107fcf49"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4917,9 +4628,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B0F4E8F-EADE-4687-BD92-9F44E749F726}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E29F4A5-09ED-4CF7-BCF2-7F7E65809C74}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c1ca76c8-b577-4424-b1c5-5c92107fcf49"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>